<commit_message>
Updated example data. Fixed broken link in readme, re-ran with newest version, including first level results in 5mm & 12mm (not just Orig & Norm SC XLS)
</commit_message>
<xml_diff>
--- a/example data/group/PCA Feature Summary.xlsx
+++ b/example data/group/PCA Feature Summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,525 +459,1715 @@
           <t>PC 3 Value</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>PC 4 Features</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>PC 4 Value</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>PC 5 Features</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>PC 5 Value</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>PC 6 Features</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>PC 6 Value</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>PC 7 Features</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>PC 7 Value</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>PC 8 Features</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>PC 8 Value</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>PC 9 Features</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>PC 9 Value</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>PC 10 Features</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>PC 10 Value</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Hind paw tao y 32</t>
+          <t>Elbow x 72</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.1342464435884682</v>
+        <v>0.05398302603340436</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Hip Angle 36</t>
+          <t>Hind paw tao y 24</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.153912465925121</v>
+        <v>0.06324021534947404</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Knee y 36</t>
+          <t>Ankle Angle Velocity 52</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.1818768059637232</v>
+        <v>0.07191163405843838</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 20</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>0.07994956482311939</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 100</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0.09536847152662994</v>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Ankle Acceleration 28</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>0.1045369595225626</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Hip Angle Velocity 92</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0.09952501710318495</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 52</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>0.1360348642848157</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 64</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>0.1182390297400654</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 72</t>
+        </is>
+      </c>
+      <c r="T2" t="n">
+        <v>0.1345508138083081</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hind paw tao y 48</t>
+          <t>Elbow x 68</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.1336389540234381</v>
+        <v>0.05393898652051591</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Hip Angle 40</t>
+          <t>Elbow y 48</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.1530404710210445</v>
+        <v>0.06263649788983566</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Knee y 32</t>
+          <t>Knee Angle Acceleration 40</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.1764582628887761</v>
+        <v>0.06780966149324963</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 16</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>0.07746867782112622</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 100</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0.09491997714629774</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Ankle Angle Velocity 24</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>-0.1016973973974226</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Ankle Acceleration 100</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>0.09653241541770062</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 52</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>0.1221670266091603</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 4</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>0.10491677882494</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 72</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>-0.1345420736179859</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Hind paw tao y 60</t>
+          <t>Elbow x 64</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.1313145008513997</v>
+        <v>0.05388494262698297</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Hip Angle 32</t>
+          <t>Elbow y 44</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.146658414273588</v>
+        <v>0.06157443363284676</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Knee y 28</t>
+          <t>Hip Angle 8</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.1730109883588847</v>
+        <v>-0.06780232119766359</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 24</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>0.0757322740669981</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Ankle Angle 40</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0.09394409461857113</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Ankle Angle Acceleration 28</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>0.09873097225193612</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 60</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>0.09311399462693294</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Ankle Acceleration 68</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>-0.1136954275121474</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 4</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>-0.1041832884452429</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>Ankle Angle Acceleration 68</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>0.1293769928104806</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hind paw tao y 44</t>
+          <t>Upper Shoulder x 72</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1304628256512615</v>
+        <v>0.05370381714711218</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Knee Angle 4</t>
+          <t>Elbow y 52</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.1461663306478759</v>
+        <v>0.06154938213060782</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Knee y 40</t>
+          <t>Elbow y 8</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.1713642347183294</v>
+        <v>0.06573595118136044</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 8</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>0.07290369004519232</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Ankle Angle 56</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0.09082303734125362</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Ear base y 100</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>-0.09708256700548333</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Ankle Acceleration 96</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>0.09311131800983473</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Ankle Acceleration 8</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>0.1122324165817821</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Hip Angle Acceleration 60</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>-0.1023127091163708</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 60</t>
+        </is>
+      </c>
+      <c r="T5" t="n">
+        <v>0.1204813785662331</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Hind paw tao y 64</t>
+          <t>Iliac Crest x 48</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.1303627029653808</v>
+        <v>0.05364785356056875</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Knee Angle 84</t>
+          <t>Hind paw tao y 20</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.1446045087597676</v>
+        <v>0.06023328813961587</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Knee y 24</t>
+          <t>Ear base y 88</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.1688470961064404</v>
+        <v>0.06571509428424306</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 84</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>0.07274435930853497</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Knee Angle 36</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0.09024873496778023</v>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 28</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>0.09114067513319672</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>Hip Angle Acceleration 88</t>
+        </is>
+      </c>
+      <c r="N6" t="n">
+        <v>0.09211938676401485</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Hip Angle Acceleration 100</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>0.1108442679859337</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 68</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>0.09662229818501586</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>Hip Angle Acceleration 72</t>
+        </is>
+      </c>
+      <c r="T6" t="n">
+        <v>-0.1192083686630647</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hind paw tao y 28</t>
+          <t>Iliac Crest x 52</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1301027350988425</v>
+        <v>0.05361370155454965</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Knee Angle 88</t>
+          <t>Hip Velocity 80</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.14457377425394</v>
+        <v>0.06017893842606759</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Knee Angle 36</t>
+          <t>Front paw tao y 44</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.1629769378572201</v>
+        <v>0.06555996437413586</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 80</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>0.07262390334887618</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ankle Angle 44</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0.08998021007620212</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Ankle Angle Acceleration 32</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>0.09037887021111225</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Hip Angle Acceleration 80</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>-0.09096960954995728</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 28</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>-0.106720002581361</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 24</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>0.09651077938805999</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 20</t>
+        </is>
+      </c>
+      <c r="T7" t="n">
+        <v>0.1142699532161501</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Hind paw tao y 52</t>
+          <t>Lower Shoulder x 60</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.1290013654368963</v>
+        <v>0.05353255379061813</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Knee Angle 80</t>
+          <t>Front paw tao y 80</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.1416345469818588</v>
+        <v>0.05937944995605245</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Knee Angle 40</t>
+          <t>Hip Angle 12</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.1609238513777707</v>
+        <v>-0.06520666342423952</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 76</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>0.07240038136441851</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Ankle Angle 52</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0.08959242272440228</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 28</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>0.08846884103937622</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 80</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>-0.09056856259513578</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 4</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>0.1051110472496437</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Ankle Angle 4</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>0.09449145403390814</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>Ankle Angle Acceleration 12</t>
+        </is>
+      </c>
+      <c r="T8" t="n">
+        <v>-0.1107552863115432</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hind paw tao y 56</t>
+          <t>Iliac Crest x 44</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.1283354967203774</v>
+        <v>0.05348859149164299</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hip Angle 44</t>
+          <t>Elbow y 40</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.140736832614998</v>
+        <v>0.05921833338925185</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Knee y 44</t>
+          <t>Front paw tao y 40</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.1602919791396059</v>
+        <v>0.06489305927049817</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Hip y 84</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>0.07159033137813327</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Knee Angle 44</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0.08926649015556133</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Nose y 28</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>-0.0880871626493924</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Knee Angle Velocity 100</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>-0.08987031099903396</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 100</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>-0.1050198688818637</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 12</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>-0.09394173408358288</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 76</t>
+        </is>
+      </c>
+      <c r="T9" t="n">
+        <v>-0.1081940119468741</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Hind paw tao y 40</t>
+          <t>Upper Shoulder x 76</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.1278902308121446</v>
+        <v>0.05346691426322678</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Knee Angle 100</t>
+          <t>Hind paw tao y 32</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.1398901607862666</v>
+        <v>0.05909723965970348</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Knee y 20</t>
+          <t>Knee Angle Velocity 36</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.1512814615103148</v>
+        <v>-0.0648194550983477</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 72</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>0.07144105395609456</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Knee Angle 40</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0.08849686338695359</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 88</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>0.08681269906938238</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Ankle Velocity 100</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>0.0877775466844946</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Hind paw tao Acceleration 100</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>-0.1038501546715625</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Ankle Acceleration 16</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>-0.09215712213316403</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 60</t>
+        </is>
+      </c>
+      <c r="T10" t="n">
+        <v>0.1079965221498587</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Hind paw tao y 68</t>
+          <t>Upper Shoulder x 68</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.1269665530884869</v>
+        <v>0.05345492706717524</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Knee Angle 76</t>
+          <t>Lower Shoulder y 48</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.1395526155306649</v>
+        <v>0.05905089056321801</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Knee y 8</t>
+          <t>Elbow y 12</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.1444320050229158</v>
+        <v>0.06391716961269281</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 4</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>0.07140127333247841</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Knee Angle 32</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0.08834616005847705</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Nose y 40</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>-0.08640978428562784</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 80</t>
+        </is>
+      </c>
+      <c r="N11" t="n">
+        <v>-0.08550862765614423</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 64</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>-0.1034687254713715</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 64</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>0.09215588961553556</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>Nose y 84</t>
+        </is>
+      </c>
+      <c r="T11" t="n">
+        <v>0.1079105260497317</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hind paw tao y 76</t>
+          <t>Iliac Crest x 56</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.1261683979824902</v>
+        <v>0.05342981501073413</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Hip Angle 28</t>
+          <t>Elbow y 56</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.1378984168789012</v>
+        <v>0.05901157252601748</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Knee Angle 44</t>
+          <t>Hip Velocity 48</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.1442799855396353</v>
+        <v>-0.0633959298225882</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 96</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>0.07138440225932234</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Knee Angle 48</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0.08833011500016917</v>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 8</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>-0.08528767527063418</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 96</t>
+        </is>
+      </c>
+      <c r="N12" t="n">
+        <v>-0.08505236181532207</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Hind paw tao Velocity 100</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>-0.1015480105927919</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 16</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>-0.08947023180940335</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>Hind paw tao Acceleration 4</t>
+        </is>
+      </c>
+      <c r="T12" t="n">
+        <v>-0.1025411757127939</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Hind paw tao y 36</t>
+          <t>Elbow x 76</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.1259626611536804</v>
+        <v>0.05340208505182547</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hip Angle 20</t>
+          <t>Hind paw tao y 28</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.1353714123444325</v>
+        <v>0.05871614115779129</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Hip Angle 92</t>
+          <t>Elbow y 20</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.1424007408530125</v>
+        <v>0.0632513030830521</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 100</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>0.07120064053697918</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Ankle Angle Velocity 64</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>-0.08812854260083312</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Hip Angle Velocity 64</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>0.08368513349316929</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Hip Angle Velocity 32</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>-0.08479227093374925</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Hip Angle Velocity 100</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>0.1012308007428754</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Hind paw tao Acceleration 56</t>
+        </is>
+      </c>
+      <c r="R13" t="n">
+        <v>-0.08937905155176809</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Ankle Angle 4</t>
+        </is>
+      </c>
+      <c r="T13" t="n">
+        <v>-0.1007034023311633</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Hind paw tao y 72</t>
+          <t>Upper Shoulder x 64</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.1256301019630757</v>
+        <v>0.05328344666497805</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hip Angle 24</t>
+          <t>Iliac Crest Velocity 80</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.1353705408894048</v>
+        <v>0.05799005457723217</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Knee y 48</t>
+          <t>Elbow y 24</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.1413290228940638</v>
+        <v>0.06323401942209103</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 28</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>0.07099648572811332</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Ankle Angle 48</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0.08454318712208071</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 64</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>0.08321233717101427</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 8</t>
+        </is>
+      </c>
+      <c r="N14" t="n">
+        <v>-0.08432414638646556</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Iliac Crest Velocity 8</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>0.09981985239274557</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Ankle Angle Acceleration 4</t>
+        </is>
+      </c>
+      <c r="R14" t="n">
+        <v>-0.08828967220485917</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Nose x 92</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>0.09926034695541974</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Hind paw tao y 80</t>
+          <t>Elbow x 60</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1232675276832881</v>
+        <v>0.05324271027674359</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Knee Angle 92</t>
+          <t>Lower Shoulder y 52</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.134707338328118</v>
+        <v>0.05797299561587465</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Knee Angle 48</t>
+          <t>Elbow y 4</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.1374327757521246</v>
+        <v>0.06228516616764635</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Hip y 28</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>0.07099047005598325</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 16</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>-0.0830207109590102</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Hip Velocity 4</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>0.08216247475368525</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 100</t>
+        </is>
+      </c>
+      <c r="N15" t="n">
+        <v>-0.08389513865189484</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 100</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>0.09910467858628091</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 60</t>
+        </is>
+      </c>
+      <c r="R15" t="n">
+        <v>0.08619939066437059</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 40</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>-0.09883501297721488</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Hind paw tao y 24</t>
+          <t>Hip x 52</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.120313775716553</v>
+        <v>0.05319545564918723</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ankle y 40</t>
+          <t>Knee y 52</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.1325016494155733</v>
+        <v>0.05790141379377651</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Knee Angle 32</t>
+          <t>Knee Angle Acceleration 44</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.1370415901641198</v>
+        <v>0.06145097787219255</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 88</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>0.07055709983749674</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Knee Angle 52</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0.08208524844328786</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 56</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>0.08121110912538695</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Knee Angle Velocity 8</t>
+        </is>
+      </c>
+      <c r="N16" t="n">
+        <v>-0.08052852892396567</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Nose x 68</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>-0.09756795951870438</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Iliac Crest Velocity 4</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>0.08507389289251625</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Hip Angle Acceleration 76</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>0.09758736872364461</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Knee y 72</t>
+          <t>Knee x 44</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.1156987996537894</v>
+        <v>0.05319470845188427</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Knee Angle 8</t>
+          <t>Upper Shoulder y 48</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.132207756098263</v>
+        <v>0.05779788132029847</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Knee y 12</t>
+          <t>Ear base y 60</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.135411889431987</v>
+        <v>0.06143587678167629</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Hip y 24</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>0.07045242265341876</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Ankle Angle Velocity 68</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>-0.08064948077151518</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Nose y 44</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>-0.08115329373106568</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Knee Angle Velocity 92</t>
+        </is>
+      </c>
+      <c r="N17" t="n">
+        <v>0.07838988318418164</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Ankle Angle 96</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>-0.09430820129487553</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 68</t>
+        </is>
+      </c>
+      <c r="R17" t="n">
+        <v>-0.08493749120220226</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 32</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>0.09758640281115386</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Knee y 76</t>
+          <t>Iliac Crest x 68</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.1149734588655372</v>
+        <v>0.05316091614912955</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Knee Angle 96</t>
+          <t>Hind paw tao y 36</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.1319469849972985</v>
+        <v>0.05766833809802148</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Knee Angle 56</t>
+          <t>Wrist y 20</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.1308818850297294</v>
+        <v>0.06091026899112804</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Iliac Crest y 12</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>0.0704314882744089</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Ankle Angle 36</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0.08031258932105509</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Nose y 32</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>-0.0791021972290331</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Nose y 84</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>0.07751606699486209</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Nose x 80</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>-0.09429197758624498</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Knee Angle Acceleration 60</t>
+        </is>
+      </c>
+      <c r="R18" t="n">
+        <v>-0.08473549701004832</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Knee Acceleration 60</t>
+        </is>
+      </c>
+      <c r="T18" t="n">
+        <v>0.09585745433818312</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Knee y 68</t>
+          <t>Hip x 44</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.1147505810726003</v>
+        <v>0.05311592282279364</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ankle y 4</t>
+          <t>Ankle y 12</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>-0.1291905490036921</v>
+        <v>0.05763468692970019</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Knee Angle 28</t>
+          <t>Wrist y 32</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.1299166805524231</v>
+        <v>0.06073370723676566</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Knee Angle 20</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>0.0700114601008491</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Ankle Angle 60</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>0.07856576146106602</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Nose y 36</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>-0.07883372782165951</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Hip Acceleration 72</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>0.07747584957878507</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Nose x 88</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>-0.09332706628224723</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Iliac Crest Acceleration 68</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>0.08442659166209708</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Hip Angle Acceleration 48</t>
+        </is>
+      </c>
+      <c r="T19" t="n">
+        <v>-0.09411370243043947</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Knee y 64</t>
+          <t>Knee x 40</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.1146787559610112</v>
+        <v>0.05306402173415975</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Ankle y 36</t>
+          <t>Knee y 56</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.1284113475117321</v>
+        <v>0.05752757817345189</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Knee Angle 52</t>
+          <t>Ear base y 44</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.1297604979051416</v>
+        <v>0.06067821132757267</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Hip y 32</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>0.06959070857271356</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Ankle Angle Velocity 72</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>-0.07698124722749672</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Nose y 24</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>-0.07754326185887084</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Knee Angle Velocity 40</t>
+        </is>
+      </c>
+      <c r="N20" t="n">
+        <v>0.07704568096546427</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Nose x 76</t>
+        </is>
+      </c>
+      <c r="P20" t="n">
+        <v>-0.09305542695143756</v>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>Nose x 72</t>
+        </is>
+      </c>
+      <c r="R20" t="n">
+        <v>0.08316156084794885</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>Ankle Angle 96</t>
+        </is>
+      </c>
+      <c r="T20" t="n">
+        <v>-0.09283096836579478</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Knee y 60</t>
+          <t>Upper Shoulder x 80</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.1121718211148835</v>
+        <v>0.05302922557402438</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Knee Angle 72</t>
+          <t>Upper Shoulder y 44</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.1280476998030622</v>
+        <v>0.05751596064026169</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Hip Angle 96</t>
+          <t>Elbow y 16</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.1295461729892732</v>
+        <v>0.06062656503039656</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Nose y 96</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>-0.0695788606026549</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Ankle Angle Velocity 76</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>-0.0765849710162344</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Hip Angle Velocity 92</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>-0.07752631395412284</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Knee Angle 96</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>0.07662355171631705</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Nose x 72</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>-0.09298266753015504</v>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>Hip Angle Acceleration 68</t>
+        </is>
+      </c>
+      <c r="R21" t="n">
+        <v>0.08153118793945671</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Ankle Angle 100</t>
+        </is>
+      </c>
+      <c r="T21" t="n">
+        <v>-0.08951529269046866</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed wrong example group names making tests fail. also reduced 5mm and 12mm results foldersto only orig & norm SC XLS fiels to limit repo size. also updated example data link and added it to main readme too
</commit_message>
<xml_diff>
--- a/example data/group/PCA Feature Summary.xlsx
+++ b/example data/group/PCA Feature Summary.xlsx
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05398302603340436</v>
+        <v>0.05398302603340437</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.06324021534947404</v>
+        <v>0.06324021534947402</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.07191163405843838</v>
+        <v>0.07191163405843833</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.07994956482311939</v>
+        <v>0.07994956482311925</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -569,7 +569,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.09536847152662994</v>
+        <v>0.09536847152663003</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0.1045369595225626</v>
+        <v>0.1045369595225625</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0.09952501710318495</v>
+        <v>0.09952501710318609</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.1360348642848157</v>
+        <v>0.1360348642848151</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -609,7 +609,7 @@
         </is>
       </c>
       <c r="T2" t="n">
-        <v>0.1345508138083081</v>
+        <v>0.1345508138083082</v>
       </c>
     </row>
     <row r="3">
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05393898652051591</v>
+        <v>0.05393898652051593</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.06263649788983566</v>
+        <v>0.06263649788983561</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.06780966149324963</v>
+        <v>0.06780966149324968</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.07746867782112622</v>
+        <v>0.07746867782112607</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.09491997714629774</v>
+        <v>0.09491997714629778</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>-0.1016973973974226</v>
+        <v>-0.1016973973974225</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>0.09653241541770062</v>
+        <v>0.0965324154177012</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.1221670266091603</v>
+        <v>0.1221670266091601</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>-0.1345420736179859</v>
+        <v>-0.1345420736179861</v>
       </c>
     </row>
     <row r="4">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.05388494262698297</v>
+        <v>0.05388494262698299</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.06157443363284676</v>
+        <v>0.06157443363284671</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.06780232119766359</v>
+        <v>-0.06780232119766362</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.0757322740669981</v>
+        <v>0.07573227406699803</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.09394409461857113</v>
+        <v>0.09394409461857123</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.09873097225193612</v>
+        <v>0.09873097225193611</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>0.09311399462693294</v>
+        <v>0.09311399462693329</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>-0.1136954275121474</v>
+        <v>-0.1136954275121483</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="R4" t="n">
-        <v>-0.1041832884452429</v>
+        <v>-0.1041832884452428</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>0.1293769928104806</v>
+        <v>0.1293769928104803</v>
       </c>
     </row>
     <row r="5">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.05370381714711218</v>
+        <v>0.05370381714711221</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.06154938213060782</v>
+        <v>0.0615493821306078</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.06573595118136044</v>
+        <v>0.06573595118136046</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.07290369004519232</v>
+        <v>0.07290369004519216</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.09082303734125362</v>
+        <v>0.09082303734125369</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>-0.09708256700548333</v>
+        <v>-0.09708256700548293</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>0.09311131800983473</v>
+        <v>0.09311131800983391</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.1122324165817821</v>
+        <v>0.1122324165817807</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>-0.1023127091163708</v>
+        <v>-0.1023127091163711</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>0.1204813785662331</v>
+        <v>0.1204813785662329</v>
       </c>
     </row>
     <row r="6">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.05364785356056875</v>
+        <v>0.05364785356056876</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.06023328813961587</v>
+        <v>0.06023328813961582</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.06571509428424306</v>
+        <v>0.06571509428424314</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.07274435930853497</v>
+        <v>0.0727443593085348</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.09024873496778023</v>
+        <v>0.09024873496778033</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0.09114067513319672</v>
+        <v>0.09114067513319617</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>0.09211938676401485</v>
+        <v>0.09211938676401597</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.1108442679859337</v>
+        <v>0.1108442679859319</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="R6" t="n">
-        <v>0.09662229818501586</v>
+        <v>0.09662229818501598</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>-0.1192083686630647</v>
+        <v>-0.1192083686630648</v>
       </c>
     </row>
     <row r="7">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.06017893842606759</v>
+        <v>0.06017893842606764</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.06555996437413586</v>
+        <v>0.06555996437413587</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.07262390334887618</v>
+        <v>0.07262390334887599</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.08998021007620212</v>
+        <v>0.08998021007620219</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0.09037887021111225</v>
+        <v>0.09037887021111257</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>-0.09096960954995728</v>
+        <v>-0.09096960954995785</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>-0.106720002581361</v>
+        <v>-0.1067200025813614</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>0.09651077938805999</v>
+        <v>0.09651077938805984</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="T7" t="n">
-        <v>0.1142699532161501</v>
+        <v>0.1142699532161502</v>
       </c>
     </row>
     <row r="8">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.05353255379061813</v>
+        <v>0.05353255379061815</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.05937944995605245</v>
+        <v>0.05937944995605241</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-0.06520666342423952</v>
+        <v>-0.06520666342423949</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.07240038136441851</v>
+        <v>0.07240038136441833</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.08959242272440228</v>
+        <v>0.0895924227244024</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0.08846884103937622</v>
+        <v>0.08846884103937577</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>-0.09056856259513578</v>
+        <v>-0.09056856259513446</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>0.09449145403390814</v>
+        <v>0.09449145403390834</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="T8" t="n">
-        <v>-0.1107552863115432</v>
+        <v>-0.1107552863115431</v>
       </c>
     </row>
     <row r="9">
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.05348859149164299</v>
+        <v>0.05348859149164303</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.05921833338925185</v>
+        <v>0.0592183333892518</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.06489305927049817</v>
+        <v>0.06489305927049822</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.07159033137813327</v>
+        <v>0.07159033137813307</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.08926649015556133</v>
+        <v>0.08926649015556143</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>-0.0880871626493924</v>
+        <v>-0.08808716264939191</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>-0.08987031099903396</v>
+        <v>-0.08987031099903621</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>-0.1050198688818637</v>
+        <v>-0.1050198688818619</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>-0.09394173408358288</v>
+        <v>-0.09394173408358301</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="T9" t="n">
-        <v>-0.1081940119468741</v>
+        <v>-0.108194011946874</v>
       </c>
     </row>
     <row r="10">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.05346691426322678</v>
+        <v>0.0534669142632268</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.05909723965970348</v>
+        <v>0.0590972396597035</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.07144105395609456</v>
+        <v>0.07144105395609436</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.08849686338695359</v>
+        <v>0.08849686338695374</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.08681269906938238</v>
+        <v>0.08681269906938253</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>0.0877775466844946</v>
+        <v>0.08777754668449492</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>-0.1038501546715625</v>
+        <v>-0.1038501546715609</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>-0.09215712213316403</v>
+        <v>-0.09215712213316399</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.05345492706717524</v>
+        <v>0.05345492706717526</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.05905089056321801</v>
+        <v>0.05905089056321794</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.06391716961269281</v>
+        <v>0.06391716961269285</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0.07140127333247841</v>
+        <v>0.07140127333247828</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.08834616005847705</v>
+        <v>0.08834616005847712</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>-0.08640978428562784</v>
+        <v>-0.0864097842856273</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>-0.08550862765614423</v>
+        <v>-0.08550862765614456</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>0.09215588961553556</v>
+        <v>0.09215588961553545</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="T11" t="n">
-        <v>0.1079105260497317</v>
+        <v>0.1079105260497316</v>
       </c>
     </row>
     <row r="12">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.05342981501073413</v>
+        <v>0.05342981501073412</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.05901157252601748</v>
+        <v>0.05901157252601743</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.0633959298225882</v>
+        <v>-0.06339592982258817</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0.07138440225932234</v>
+        <v>0.07138440225932217</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.08833011500016917</v>
+        <v>0.08833011500016932</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>-0.08528767527063418</v>
+        <v>-0.08528767527063502</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>-0.08505236181532207</v>
+        <v>-0.08505236181532355</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>-0.1015480105927919</v>
+        <v>-0.1015480105927904</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>-0.08947023180940335</v>
+        <v>-0.08947023180940337</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="T12" t="n">
-        <v>-0.1025411757127939</v>
+        <v>-0.1025411757127937</v>
       </c>
     </row>
     <row r="13">
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>0.05340208505182547</v>
+        <v>0.05340208505182548</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.05871614115779129</v>
+        <v>0.05871614115779131</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.0632513030830521</v>
+        <v>0.06325130308305212</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.07120064053697918</v>
+        <v>0.07120064053697901</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>-0.08812854260083312</v>
+        <v>-0.08812854260083321</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>0.08368513349316929</v>
+        <v>0.08368513349316971</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>-0.08479227093374925</v>
+        <v>-0.08479227093375025</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.1012308007428754</v>
+        <v>0.1012308007428736</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="T13" t="n">
-        <v>-0.1007034023311633</v>
+        <v>-0.1007034023311632</v>
       </c>
     </row>
     <row r="14">
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.05328344666497805</v>
+        <v>0.05328344666497807</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.05799005457723217</v>
+        <v>0.0579900545772322</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.06323401942209103</v>
+        <v>0.06323401942209098</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.07099648572811332</v>
+        <v>0.07099648572811322</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0.08454318712208071</v>
+        <v>0.0845431871220808</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>0.08321233717101427</v>
+        <v>0.08321233717101384</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1569,7 +1569,7 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>-0.08432414638646556</v>
+        <v>-0.08432414638646449</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.09981985239274557</v>
+        <v>0.09981985239274546</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="T14" t="n">
-        <v>0.09926034695541974</v>
+        <v>0.09926034695541948</v>
       </c>
     </row>
     <row r="15">
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.05797299561587465</v>
+        <v>0.05797299561587459</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.06228516616764635</v>
+        <v>0.06228516616764638</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.07099047005598325</v>
+        <v>0.07099047005598309</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>-0.0830207109590102</v>
+        <v>-0.08302071095901038</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>0.08216247475368525</v>
+        <v>0.082162474753686</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>-0.08389513865189484</v>
+        <v>-0.08389513865189718</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.09910467858628091</v>
+        <v>0.0991046785862788</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>0.08619939066437059</v>
+        <v>0.08619939066437048</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="T15" t="n">
-        <v>-0.09883501297721488</v>
+        <v>-0.09883501297721461</v>
       </c>
     </row>
     <row r="16">
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.05319545564918723</v>
+        <v>0.05319545564918726</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.05790141379377651</v>
+        <v>0.0579014137937765</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.06145097787219255</v>
+        <v>0.06145097787219245</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1709,7 +1709,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.07055709983749674</v>
+        <v>0.0705570998374965</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0.08208524844328786</v>
+        <v>0.08208524844328799</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>0.08121110912538695</v>
+        <v>0.08121110912538704</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>-0.08052852892396567</v>
+        <v>-0.08052852892396543</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>-0.09756795951870438</v>
+        <v>-0.09756795951870498</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="R16" t="n">
-        <v>0.08507389289251625</v>
+        <v>0.0850738928925161</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="T16" t="n">
-        <v>0.09758736872364461</v>
+        <v>0.09758736872364451</v>
       </c>
     </row>
     <row r="17">
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.05319470845188427</v>
+        <v>0.05319470845188429</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.05779788132029847</v>
+        <v>0.0577978813202984</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.06143587678167629</v>
+        <v>0.06143587678167636</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.07045242265341876</v>
+        <v>0.07045242265341863</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>-0.08064948077151518</v>
+        <v>-0.08064948077151528</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>-0.08115329373106568</v>
+        <v>-0.08115329373106529</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>0.07838988318418164</v>
+        <v>0.07838988318418295</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>-0.09430820129487553</v>
+        <v>-0.09430820129487467</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>-0.08493749120220226</v>
+        <v>-0.08493749120220237</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="T17" t="n">
-        <v>0.09758640281115386</v>
+        <v>0.09758640281115397</v>
       </c>
     </row>
     <row r="18">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.05316091614912955</v>
+        <v>0.05316091614912954</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.05766833809802148</v>
+        <v>0.05766833809802152</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.06091026899112804</v>
+        <v>0.06091026899112795</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0.0704314882744089</v>
+        <v>0.07043148827440877</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.08031258932105509</v>
+        <v>0.08031258932105516</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>-0.0791021972290331</v>
+        <v>-0.07910219722903247</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>0.07751606699486209</v>
+        <v>0.07751606699486216</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>-0.09429197758624498</v>
+        <v>-0.09429197758624523</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="R18" t="n">
-        <v>-0.08473549701004832</v>
+        <v>-0.08473549701004858</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="T18" t="n">
-        <v>0.09585745433818312</v>
+        <v>0.09585745433818331</v>
       </c>
     </row>
     <row r="19">
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.05311592282279364</v>
+        <v>0.05311592282279366</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.05763468692970019</v>
+        <v>0.0576346869297002</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.06073370723676566</v>
+        <v>0.06073370723676563</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0.07856576146106602</v>
+        <v>0.07856576146106607</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>-0.07883372782165951</v>
+        <v>-0.07883372782165897</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>0.07747584957878507</v>
+        <v>0.07747584957878531</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>-0.09332706628224723</v>
+        <v>-0.09332706628224754</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>0.08442659166209708</v>
+        <v>0.08442659166209704</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="T19" t="n">
-        <v>-0.09411370243043947</v>
+        <v>-0.09411370243043944</v>
       </c>
     </row>
     <row r="20">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.05306402173415975</v>
+        <v>0.05306402173415979</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.05752757817345189</v>
+        <v>0.05752757817345187</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.06067821132757267</v>
+        <v>0.06067821132757273</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.06959070857271356</v>
+        <v>0.06959070857271345</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>-0.07698124722749672</v>
+        <v>-0.07698124722749669</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>-0.07754326185887084</v>
+        <v>-0.0775432618588703</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>0.07704568096546427</v>
+        <v>0.07704568096546437</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>-0.09305542695143756</v>
+        <v>-0.09305542695143779</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="R20" t="n">
-        <v>0.08316156084794885</v>
+        <v>0.0831615608479489</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="T20" t="n">
-        <v>-0.09283096836579478</v>
+        <v>-0.09283096836579473</v>
       </c>
     </row>
     <row r="21">
@@ -2095,7 +2095,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.05302922557402438</v>
+        <v>0.05302922557402436</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.05751596064026169</v>
+        <v>0.05751596064026161</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.06062656503039656</v>
+        <v>0.0606265650303966</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>-0.0695788606026549</v>
+        <v>-0.06957886060265482</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>-0.0765849710162344</v>
+        <v>-0.07658497101623438</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>-0.07752631395412284</v>
+        <v>-0.07752631395412193</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>0.07662355171631705</v>
+        <v>0.0766235517163172</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2151,7 +2151,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>-0.09298266753015504</v>
+        <v>-0.0929826675301553</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>0.08153118793945671</v>
+        <v>0.08153118793945698</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="T21" t="n">
-        <v>-0.08951529269046866</v>
+        <v>-0.08951529269046864</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
group approval was failing because now x-standardising and the group GUI config was different. also need to ensure pca n components is an int if >1 - added in group prep
</commit_message>
<xml_diff>
--- a/example data/group/PCA Feature Summary.xlsx
+++ b/example data/group/PCA Feature Summary.xlsx
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05398302603340437</v>
+        <v>0.05398302603340439</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.06324021534947402</v>
+        <v>0.06324021534947406</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.07191163405843833</v>
+        <v>0.07191163405843846</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.07994956482311925</v>
+        <v>0.07994956482311931</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -577,7 +577,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0.1045369595225625</v>
+        <v>0.1045369595225626</v>
       </c>
       <c r="M2" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0.09952501710318609</v>
+        <v>0.09952501710318547</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.1360348642848151</v>
+        <v>0.1360348642848153</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="R2" t="n">
-        <v>0.1182390297400654</v>
+        <v>0.1182390297400656</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05393898652051593</v>
+        <v>0.05393898652051596</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.06263649788983561</v>
+        <v>0.06263649788983572</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.06780966149324968</v>
+        <v>0.0678096614932498</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.07746867782112607</v>
+        <v>0.07746867782112618</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.09491997714629778</v>
+        <v>0.09491997714629781</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -659,7 +659,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>-0.1016973973974225</v>
+        <v>-0.1016973973974226</v>
       </c>
       <c r="M3" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>0.0965324154177012</v>
+        <v>0.09653241541770088</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.1221670266091601</v>
+        <v>0.1221670266091602</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>0.10491677882494</v>
+        <v>0.1049167788249398</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="T3" t="n">
-        <v>-0.1345420736179861</v>
+        <v>-0.1345420736179862</v>
       </c>
     </row>
     <row r="4">
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.05388494262698299</v>
+        <v>0.053884942626983</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.06157443363284671</v>
+        <v>0.06157443363284685</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.06780232119766362</v>
+        <v>-0.06780232119766368</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.07573227406699803</v>
+        <v>0.07573227406699812</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.09394409461857123</v>
+        <v>0.09394409461857124</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.09873097225193611</v>
+        <v>0.0987309722519361</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>0.09311399462693329</v>
+        <v>0.09311399462693297</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>-0.1136954275121483</v>
+        <v>-0.113695427512148</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="R4" t="n">
-        <v>-0.1041832884452428</v>
+        <v>-0.1041832884452427</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>0.1293769928104803</v>
+        <v>0.1293769928104796</v>
       </c>
     </row>
     <row r="5">
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.0615493821306078</v>
+        <v>0.06154938213060791</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.06573595118136046</v>
+        <v>0.06573595118136047</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.07290369004519216</v>
+        <v>0.07290369004519225</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -815,7 +815,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>0.09082303734125369</v>
+        <v>0.09082303734125366</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>-0.09708256700548293</v>
+        <v>-0.09708256700548316</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>0.09311131800983391</v>
+        <v>0.09311131800983408</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.1122324165817807</v>
+        <v>0.1122324165817813</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>-0.1023127091163711</v>
+        <v>-0.102312709116371</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="T5" t="n">
-        <v>0.1204813785662329</v>
+        <v>0.1204813785662333</v>
       </c>
     </row>
     <row r="6">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.05364785356056876</v>
+        <v>0.05364785356056877</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.06023328813961582</v>
+        <v>0.06023328813961594</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.06571509428424314</v>
+        <v>0.0657150942842431</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.0727443593085348</v>
+        <v>0.07274435930853486</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.09024873496778033</v>
+        <v>0.09024873496778038</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0.09114067513319617</v>
+        <v>0.09114067513319668</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>0.09211938676401597</v>
+        <v>0.09211938676401549</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.1108442679859319</v>
+        <v>0.1108442679859327</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="R6" t="n">
-        <v>0.09662229818501598</v>
+        <v>0.09662229818501593</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>-0.1192083686630648</v>
+        <v>-0.1192083686630658</v>
       </c>
     </row>
     <row r="7">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.05361370155454965</v>
+        <v>0.05361370155454967</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.06017893842606764</v>
+        <v>0.06017893842606765</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.06555996437413587</v>
+        <v>0.06555996437413589</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.07262390334887599</v>
+        <v>0.07262390334887613</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.08998021007620219</v>
+        <v>0.08998021007620215</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0.09037887021111257</v>
+        <v>0.09037887021111249</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>-0.09096960954995785</v>
+        <v>-0.09096960954995778</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>-0.1067200025813614</v>
+        <v>-0.1067200025813611</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>0.09651077938805984</v>
+        <v>0.09651077938805969</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="T7" t="n">
-        <v>0.1142699532161502</v>
+        <v>0.1142699532161501</v>
       </c>
     </row>
     <row r="8">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.05353255379061815</v>
+        <v>0.05353255379061816</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.05937944995605241</v>
+        <v>0.05937944995605254</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-0.06520666342423949</v>
+        <v>-0.06520666342423959</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.07240038136441833</v>
+        <v>0.07240038136441847</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.0895924227244024</v>
+        <v>0.08959242272440235</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0.08846884103937577</v>
+        <v>0.08846884103937622</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>-0.09056856259513446</v>
+        <v>-0.09056856259513471</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.1051110472496437</v>
+        <v>0.1051110472496439</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>0.09449145403390834</v>
+        <v>0.09449145403390842</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1101,7 +1101,7 @@
         </is>
       </c>
       <c r="T8" t="n">
-        <v>-0.1107552863115431</v>
+        <v>-0.1107552863115432</v>
       </c>
     </row>
     <row r="9">
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.05348859149164303</v>
+        <v>0.05348859149164301</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.0592183333892518</v>
+        <v>0.05921833338925195</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.06489305927049822</v>
+        <v>0.06489305927049821</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.07159033137813307</v>
+        <v>0.07159033137813312</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.08926649015556143</v>
+        <v>0.08926649015556147</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>-0.08808716264939191</v>
+        <v>-0.08808716264939202</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>-0.08987031099903621</v>
+        <v>-0.08987031099903553</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>-0.1050198688818619</v>
+        <v>-0.1050198688818627</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>-0.09394173408358301</v>
+        <v>-0.09394173408358299</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="T9" t="n">
-        <v>-0.108194011946874</v>
+        <v>-0.1081940119468742</v>
       </c>
     </row>
     <row r="10">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.0534669142632268</v>
+        <v>0.05346691426322681</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.0590972396597035</v>
+        <v>0.05909723965970352</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>-0.0648194550983477</v>
+        <v>-0.06481945509834784</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.07144105395609436</v>
+        <v>0.0714410539560945</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.08849686338695374</v>
+        <v>0.0884968633869537</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.08681269906938253</v>
+        <v>0.0868126990693822</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>0.08777754668449492</v>
+        <v>0.08777754668449493</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>-0.1038501546715609</v>
+        <v>-0.1038501546715616</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>-0.09215712213316399</v>
+        <v>-0.09215712213316382</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1265,7 +1265,7 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>0.1079965221498587</v>
+        <v>0.1079965221498594</v>
       </c>
     </row>
     <row r="11">
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.05905089056321794</v>
+        <v>0.05905089056321808</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.06391716961269285</v>
+        <v>0.06391716961269286</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0.07140127333247828</v>
+        <v>0.07140127333247835</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.08834616005847712</v>
+        <v>0.08834616005847719</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>-0.0864097842856273</v>
+        <v>-0.08640978428562747</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>-0.08550862765614456</v>
+        <v>-0.08550862765614455</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>-0.1034687254713715</v>
+        <v>-0.1034687254713713</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>0.09215588961553545</v>
+        <v>0.09215588961553586</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="T11" t="n">
-        <v>0.1079105260497316</v>
+        <v>0.1079105260497315</v>
       </c>
     </row>
     <row r="12">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.05342981501073412</v>
+        <v>0.05342981501073413</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.05901157252601743</v>
+        <v>0.05901157252601754</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.06339592982258817</v>
+        <v>-0.06339592982258822</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1381,7 +1381,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>0.07138440225932217</v>
+        <v>0.0713844022593223</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.08833011500016932</v>
+        <v>0.08833011500016925</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>-0.08528767527063502</v>
+        <v>-0.08528767527063447</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>-0.08505236181532355</v>
+        <v>-0.08505236181532305</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>-0.1015480105927904</v>
+        <v>-0.1015480105927911</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>-0.08947023180940337</v>
+        <v>-0.08947023180940358</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="T12" t="n">
-        <v>-0.1025411757127937</v>
+        <v>-0.1025411757127936</v>
       </c>
     </row>
     <row r="13">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.05871614115779131</v>
+        <v>0.05871614115779134</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.06325130308305212</v>
+        <v>0.06325130308305216</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.07120064053697901</v>
+        <v>0.07120064053697911</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>-0.08812854260083321</v>
+        <v>-0.08812854260083319</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>0.08368513349316971</v>
+        <v>0.08368513349316935</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>-0.08479227093375025</v>
+        <v>-0.08479227093375005</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.1012308007428736</v>
+        <v>0.1012308007428744</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>-0.08937905155176809</v>
+        <v>-0.08937905155176799</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="T13" t="n">
-        <v>-0.1007034023311632</v>
+        <v>-0.100703402331163</v>
       </c>
     </row>
     <row r="14">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.0579900545772322</v>
+        <v>0.05799005457723225</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.06323401942209098</v>
+        <v>0.06323401942209099</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>0.07099648572811322</v>
+        <v>0.0709964857281133</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0.0845431871220808</v>
+        <v>0.08454318712208073</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>0.08321233717101384</v>
+        <v>0.08321233717101427</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1569,7 +1569,7 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>-0.08432414638646449</v>
+        <v>-0.08432414638646493</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.09981985239274546</v>
+        <v>0.09981985239274575</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="R14" t="n">
-        <v>-0.08828967220485917</v>
+        <v>-0.08828967220485907</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="T14" t="n">
-        <v>0.09926034695541948</v>
+        <v>0.09926034695541949</v>
       </c>
     </row>
     <row r="15">
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.05324271027674359</v>
+        <v>0.05324271027674361</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.05797299561587459</v>
+        <v>0.05797299561587472</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.06228516616764638</v>
+        <v>0.0622851661676464</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>0.07099047005598309</v>
+        <v>0.07099047005598315</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>-0.08302071095901038</v>
+        <v>-0.0830207109590103</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>0.082162474753686</v>
+        <v>0.08216247475368543</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>-0.08389513865189718</v>
+        <v>-0.08389513865189659</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.0991046785862788</v>
+        <v>0.09910467858627972</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>0.08619939066437048</v>
+        <v>0.08619939066437056</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="T15" t="n">
-        <v>-0.09883501297721461</v>
+        <v>-0.09883501297721427</v>
       </c>
     </row>
     <row r="16">
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.0579014137937765</v>
+        <v>0.05790141379377656</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.06145097787219245</v>
+        <v>0.06145097787219254</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1709,7 +1709,7 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.0705570998374965</v>
+        <v>0.07055709983749663</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0.08208524844328799</v>
+        <v>0.08208524844328795</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>0.08121110912538704</v>
+        <v>0.08121110912538702</v>
       </c>
       <c r="M16" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>-0.08052852892396543</v>
+        <v>-0.08052852892396567</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>-0.09756795951870498</v>
+        <v>-0.09756795951870462</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="R16" t="n">
-        <v>0.0850738928925161</v>
+        <v>0.08507389289251595</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="T16" t="n">
-        <v>0.09758736872364451</v>
+        <v>0.09758736872364442</v>
       </c>
     </row>
     <row r="17">
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.05319470845188429</v>
+        <v>0.05319470845188428</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.0577978813202984</v>
+        <v>0.05779788132029856</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.06143587678167636</v>
+        <v>0.06143587678167639</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.07045242265341863</v>
+        <v>0.07045242265341869</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>-0.08064948077151528</v>
+        <v>-0.08064948077151525</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>-0.08115329373106529</v>
+        <v>-0.08115329373106532</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>0.07838988318418295</v>
+        <v>0.07838988318418236</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>-0.09430820129487467</v>
+        <v>-0.09430820129487491</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>-0.08493749120220237</v>
+        <v>-0.08493749120220222</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="T17" t="n">
-        <v>0.09758640281115397</v>
+        <v>0.09758640281115422</v>
       </c>
     </row>
     <row r="18">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.05316091614912954</v>
+        <v>0.05316091614912957</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.06091026899112795</v>
+        <v>0.06091026899112802</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0.07043148827440877</v>
+        <v>0.07043148827440883</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.08031258932105516</v>
+        <v>0.0803125893210552</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>-0.07910219722903247</v>
+        <v>-0.07910219722903268</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>0.07751606699486216</v>
+        <v>0.0775160669948621</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>-0.09429197758624523</v>
+        <v>-0.09429197758624501</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="R18" t="n">
-        <v>-0.08473549701004858</v>
+        <v>-0.08473549701004859</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="T18" t="n">
-        <v>0.09585745433818331</v>
+        <v>0.09585745433818413</v>
       </c>
     </row>
     <row r="19">
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.05311592282279366</v>
+        <v>0.05311592282279368</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.0576346869297002</v>
+        <v>0.05763468692970023</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.06073370723676563</v>
+        <v>0.06073370723676565</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>0.0700114601008491</v>
+        <v>0.07001146010084915</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0.07856576146106607</v>
+        <v>0.07856576146106603</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>-0.07883372782165897</v>
+        <v>-0.07883372782165911</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>0.07747584957878531</v>
+        <v>0.07747584957878532</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>-0.09332706628224754</v>
+        <v>-0.09332706628224716</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="T19" t="n">
-        <v>-0.09411370243043944</v>
+        <v>-0.09411370243043991</v>
       </c>
     </row>
     <row r="20">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.05306402173415979</v>
+        <v>0.05306402173415983</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.05752757817345187</v>
+        <v>0.05752757817345197</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.06959070857271345</v>
+        <v>0.0695907085727135</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>-0.0775432618588703</v>
+        <v>-0.07754326185887049</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>0.07704568096546437</v>
+        <v>0.07704568096546446</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>-0.09305542695143779</v>
+        <v>-0.0930554269514374</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="R20" t="n">
-        <v>0.0831615608479489</v>
+        <v>0.08316156084794891</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="T20" t="n">
-        <v>-0.09283096836579473</v>
+        <v>-0.09283096836579435</v>
       </c>
     </row>
     <row r="21">
@@ -2095,7 +2095,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.05302922557402436</v>
+        <v>0.05302922557402437</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.05751596064026161</v>
+        <v>0.05751596064026176</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>-0.06957886060265482</v>
+        <v>-0.06957886060265489</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>-0.07658497101623438</v>
+        <v>-0.0765849710162344</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>-0.07752631395412193</v>
+        <v>-0.07752631395412245</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>0.0766235517163172</v>
+        <v>0.076623551716317</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2151,7 +2151,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>-0.0929826675301553</v>
+        <v>-0.09298266753015501</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>0.08153118793945698</v>
+        <v>0.08153118793945723</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="T21" t="n">
-        <v>-0.08951529269046864</v>
+        <v>-0.08951529269046801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
re-ran group analysis of example data without 3d pca vid because else approval test fails on git
</commit_message>
<xml_diff>
--- a/example data/group/PCA Feature Summary.xlsx
+++ b/example data/group/PCA Feature Summary.xlsx
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05398302603340439</v>
+        <v>0.05398302603340438</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.06324021534947406</v>
+        <v>0.06324021534947402</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -553,7 +553,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.07191163405843846</v>
+        <v>0.07191163405843824</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>0.07994956482311931</v>
+        <v>0.0799495648231193</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -569,7 +569,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>0.09536847152663003</v>
+        <v>0.09536847152662997</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0.09952501710318547</v>
+        <v>0.09952501710318529</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>0.1360348642848153</v>
+        <v>0.1360348642848156</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
@@ -601,7 +601,7 @@
         </is>
       </c>
       <c r="R2" t="n">
-        <v>0.1182390297400656</v>
+        <v>0.1182390297400653</v>
       </c>
       <c r="S2" t="inlineStr">
         <is>
@@ -619,7 +619,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.05393898652051596</v>
+        <v>0.05393898652051593</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.06263649788983572</v>
+        <v>0.06263649788983565</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.0678096614932498</v>
+        <v>0.06780966149324956</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -643,7 +643,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>0.07746867782112618</v>
+        <v>0.07746867782112613</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -651,7 +651,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>0.09491997714629781</v>
+        <v>0.09491997714629777</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -667,7 +667,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>0.09653241541770088</v>
+        <v>0.09653241541770058</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>0.1221670266091602</v>
+        <v>0.1221670266091603</v>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
@@ -683,7 +683,7 @@
         </is>
       </c>
       <c r="R3" t="n">
-        <v>0.1049167788249398</v>
+        <v>0.1049167788249403</v>
       </c>
       <c r="S3" t="inlineStr">
         <is>
@@ -701,7 +701,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.053884942626983</v>
+        <v>0.05388494262698296</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -709,7 +709,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.06157443363284685</v>
+        <v>0.06157443363284674</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -717,7 +717,7 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>-0.06780232119766368</v>
+        <v>-0.06780232119766351</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>0.07573227406699812</v>
+        <v>0.0757322740669981</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -733,7 +733,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>0.09394409461857124</v>
+        <v>0.09394409461857135</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>0.0987309722519361</v>
+        <v>0.09873097225193617</v>
       </c>
       <c r="M4" t="inlineStr">
         <is>
@@ -749,7 +749,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>0.09311399462693297</v>
+        <v>0.09311399462693296</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -757,7 +757,7 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>-0.113695427512148</v>
+        <v>-0.1136954275121476</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="R4" t="n">
-        <v>-0.1041832884452427</v>
+        <v>-0.1041832884452429</v>
       </c>
       <c r="S4" t="inlineStr">
         <is>
@@ -773,7 +773,7 @@
         </is>
       </c>
       <c r="T4" t="n">
-        <v>0.1293769928104796</v>
+        <v>0.1293769928104798</v>
       </c>
     </row>
     <row r="5">
@@ -783,7 +783,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.05370381714711221</v>
+        <v>0.0537038171471122</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -791,7 +791,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.06154938213060791</v>
+        <v>0.06154938213060779</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -799,7 +799,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.06573595118136047</v>
+        <v>0.06573595118136037</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>0.07290369004519225</v>
+        <v>0.07290369004519227</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>-0.09708256700548316</v>
+        <v>-0.09708256700548293</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>0.09311131800983408</v>
+        <v>0.09311131800983437</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -839,7 +839,7 @@
         </is>
       </c>
       <c r="P5" t="n">
-        <v>0.1122324165817813</v>
+        <v>0.1122324165817816</v>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
@@ -847,7 +847,7 @@
         </is>
       </c>
       <c r="R5" t="n">
-        <v>-0.102312709116371</v>
+        <v>-0.1023127091163709</v>
       </c>
       <c r="S5" t="inlineStr">
         <is>
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.05364785356056877</v>
+        <v>0.05364785356056875</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.06023328813961594</v>
+        <v>0.06023328813961583</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.0657150942842431</v>
+        <v>0.06571509428424306</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -889,7 +889,7 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.07274435930853486</v>
+        <v>0.07274435930853479</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -897,7 +897,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>0.09024873496778038</v>
+        <v>0.09024873496778042</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -905,7 +905,7 @@
         </is>
       </c>
       <c r="L6" t="n">
-        <v>0.09114067513319668</v>
+        <v>0.09114067513319667</v>
       </c>
       <c r="M6" t="inlineStr">
         <is>
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>0.09211938676401549</v>
+        <v>0.09211938676401511</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -921,7 +921,7 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>0.1108442679859327</v>
+        <v>0.1108442679859332</v>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
@@ -929,7 +929,7 @@
         </is>
       </c>
       <c r="R6" t="n">
-        <v>0.09662229818501593</v>
+        <v>0.09662229818501591</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -937,7 +937,7 @@
         </is>
       </c>
       <c r="T6" t="n">
-        <v>-0.1192083686630658</v>
+        <v>-0.1192083686630655</v>
       </c>
     </row>
     <row r="7">
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.05361370155454967</v>
+        <v>0.05361370155454964</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.06017893842606765</v>
+        <v>0.0601789384260676</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.06555996437413589</v>
+        <v>0.0655599643741358</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>0.07262390334887613</v>
+        <v>0.07262390334887607</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -979,7 +979,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>0.08998021007620215</v>
+        <v>0.08998021007620235</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0.09037887021111249</v>
+        <v>0.09037887021111238</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -995,7 +995,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>-0.09096960954995778</v>
+        <v>-0.09096960954995749</v>
       </c>
       <c r="O7" t="inlineStr">
         <is>
@@ -1003,7 +1003,7 @@
         </is>
       </c>
       <c r="P7" t="n">
-        <v>-0.1067200025813611</v>
+        <v>-0.1067200025813612</v>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
@@ -1011,7 +1011,7 @@
         </is>
       </c>
       <c r="R7" t="n">
-        <v>0.09651077938805969</v>
+        <v>0.09651077938806005</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="T7" t="n">
-        <v>0.1142699532161501</v>
+        <v>0.1142699532161502</v>
       </c>
     </row>
     <row r="8">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.05353255379061816</v>
+        <v>0.05353255379061812</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.05937944995605254</v>
+        <v>0.05937944995605241</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>-0.06520666342423959</v>
+        <v>-0.06520666342423939</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>0.07240038136441847</v>
+        <v>0.07240038136441843</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -1061,7 +1061,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>0.08959242272440235</v>
+        <v>0.08959242272440239</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>0.08846884103937622</v>
+        <v>0.08846884103937612</v>
       </c>
       <c r="M8" t="inlineStr">
         <is>
@@ -1077,7 +1077,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>-0.09056856259513471</v>
+        <v>-0.09056856259513535</v>
       </c>
       <c r="O8" t="inlineStr">
         <is>
@@ -1085,7 +1085,7 @@
         </is>
       </c>
       <c r="P8" t="n">
-        <v>0.1051110472496439</v>
+        <v>0.1051110472496436</v>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
@@ -1093,7 +1093,7 @@
         </is>
       </c>
       <c r="R8" t="n">
-        <v>0.09449145403390842</v>
+        <v>0.09449145403390825</v>
       </c>
       <c r="S8" t="inlineStr">
         <is>
@@ -1111,7 +1111,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.05348859149164301</v>
+        <v>0.05348859149164299</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1119,7 +1119,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.05921833338925195</v>
+        <v>0.05921833338925183</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.06489305927049821</v>
+        <v>0.06489305927049813</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1135,7 +1135,7 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>0.07159033137813312</v>
+        <v>0.07159033137813313</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -1143,7 +1143,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>0.08926649015556147</v>
+        <v>0.0892664901555615</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -1151,7 +1151,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>-0.08808716264939202</v>
+        <v>-0.08808716264939211</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -1159,7 +1159,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>-0.08987031099903553</v>
+        <v>-0.08987031099903453</v>
       </c>
       <c r="O9" t="inlineStr">
         <is>
@@ -1167,7 +1167,7 @@
         </is>
       </c>
       <c r="P9" t="n">
-        <v>-0.1050198688818627</v>
+        <v>-0.1050198688818631</v>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
         </is>
       </c>
       <c r="R9" t="n">
-        <v>-0.09394173408358299</v>
+        <v>-0.09394173408358306</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
       <c r="T9" t="n">
-        <v>-0.1081940119468742</v>
+        <v>-0.1081940119468741</v>
       </c>
     </row>
     <row r="10">
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.05346691426322681</v>
+        <v>0.0534669142632268</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.05909723965970352</v>
+        <v>0.05909723965970342</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -1209,7 +1209,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>-0.06481945509834784</v>
+        <v>-0.06481945509834756</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>0.0714410539560945</v>
+        <v>0.07144105395609444</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -1225,7 +1225,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>0.0884968633869537</v>
+        <v>0.08849686338695373</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>0.0868126990693822</v>
+        <v>0.08681269906938234</v>
       </c>
       <c r="M10" t="inlineStr">
         <is>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>0.08777754668449493</v>
+        <v>0.08777754668449465</v>
       </c>
       <c r="O10" t="inlineStr">
         <is>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="P10" t="n">
-        <v>-0.1038501546715616</v>
+        <v>-0.103850154671562</v>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
@@ -1257,7 +1257,7 @@
         </is>
       </c>
       <c r="R10" t="n">
-        <v>-0.09215712213316382</v>
+        <v>-0.09215712213316411</v>
       </c>
       <c r="S10" t="inlineStr">
         <is>
@@ -1265,7 +1265,7 @@
         </is>
       </c>
       <c r="T10" t="n">
-        <v>0.1079965221498594</v>
+        <v>0.1079965221498592</v>
       </c>
     </row>
     <row r="11">
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0.05345492706717526</v>
+        <v>0.05345492706717524</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1283,7 +1283,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.05905089056321808</v>
+        <v>0.05905089056321797</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.06391716961269286</v>
+        <v>0.06391716961269278</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1299,7 +1299,7 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>0.07140127333247835</v>
+        <v>0.07140127333247834</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -1307,7 +1307,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>0.08834616005847719</v>
+        <v>0.08834616005847716</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="L11" t="n">
-        <v>-0.08640978428562747</v>
+        <v>-0.08640978428562748</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -1323,7 +1323,7 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>-0.08550862765614455</v>
+        <v>-0.08550862765614442</v>
       </c>
       <c r="O11" t="inlineStr">
         <is>
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="P11" t="n">
-        <v>-0.1034687254713713</v>
+        <v>-0.1034687254713716</v>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="R11" t="n">
-        <v>0.09215588961553586</v>
+        <v>0.09215588961553545</v>
       </c>
       <c r="S11" t="inlineStr">
         <is>
@@ -1347,7 +1347,7 @@
         </is>
       </c>
       <c r="T11" t="n">
-        <v>0.1079105260497315</v>
+        <v>0.1079105260497316</v>
       </c>
     </row>
     <row r="12">
@@ -1357,7 +1357,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0.05342981501073413</v>
+        <v>0.0534298150107341</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.05901157252601754</v>
+        <v>0.05901157252601745</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>-0.06339592982258822</v>
+        <v>-0.06339592982258811</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>0.08833011500016925</v>
+        <v>0.08833011500016928</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1397,7 +1397,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>-0.08528767527063447</v>
+        <v>-0.08528767527063467</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -1405,7 +1405,7 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>-0.08505236181532305</v>
+        <v>-0.08505236181532244</v>
       </c>
       <c r="O12" t="inlineStr">
         <is>
@@ -1413,7 +1413,7 @@
         </is>
       </c>
       <c r="P12" t="n">
-        <v>-0.1015480105927911</v>
+        <v>-0.1015480105927915</v>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="R12" t="n">
-        <v>-0.08947023180940358</v>
+        <v>-0.08947023180940329</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -1429,7 +1429,7 @@
         </is>
       </c>
       <c r="T12" t="n">
-        <v>-0.1025411757127936</v>
+        <v>-0.1025411757127937</v>
       </c>
     </row>
     <row r="13">
@@ -1447,7 +1447,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.05871614115779134</v>
+        <v>0.05871614115779125</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.06325130308305216</v>
+        <v>0.06325130308305209</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -1463,7 +1463,7 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>0.07120064053697911</v>
+        <v>0.07120064053697905</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -1471,7 +1471,7 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>-0.08812854260083319</v>
+        <v>-0.08812854260083315</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>0.08368513349316935</v>
+        <v>0.08368513349316958</v>
       </c>
       <c r="M13" t="inlineStr">
         <is>
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>-0.08479227093375005</v>
+        <v>-0.08479227093374955</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="P13" t="n">
-        <v>0.1012308007428744</v>
+        <v>0.1012308007428749</v>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
@@ -1503,7 +1503,7 @@
         </is>
       </c>
       <c r="R13" t="n">
-        <v>-0.08937905155176799</v>
+        <v>-0.08937905155176822</v>
       </c>
       <c r="S13" t="inlineStr">
         <is>
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="T13" t="n">
-        <v>-0.100703402331163</v>
+        <v>-0.1007034023311631</v>
       </c>
     </row>
     <row r="14">
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>0.05328344666497807</v>
+        <v>0.05328344666497805</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.05799005457723225</v>
+        <v>0.05799005457723216</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.06323401942209099</v>
+        <v>0.06323401942209095</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -1553,7 +1553,7 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>0.08454318712208073</v>
+        <v>0.08454318712208084</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1561,7 +1561,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>0.08321233717101427</v>
+        <v>0.08321233717101413</v>
       </c>
       <c r="M14" t="inlineStr">
         <is>
@@ -1569,7 +1569,7 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>-0.08432414638646493</v>
+        <v>-0.0843241463864651</v>
       </c>
       <c r="O14" t="inlineStr">
         <is>
@@ -1577,7 +1577,7 @@
         </is>
       </c>
       <c r="P14" t="n">
-        <v>0.09981985239274575</v>
+        <v>0.09981985239274552</v>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="R14" t="n">
-        <v>-0.08828967220485907</v>
+        <v>-0.08828967220485928</v>
       </c>
       <c r="S14" t="inlineStr">
         <is>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="T14" t="n">
-        <v>0.09926034695541949</v>
+        <v>0.09926034695541945</v>
       </c>
     </row>
     <row r="15">
@@ -1603,7 +1603,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.05324271027674361</v>
+        <v>0.05324271027674356</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.05797299561587472</v>
+        <v>0.05797299561587464</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.0622851661676464</v>
+        <v>0.06228516616764626</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>-0.0830207109590103</v>
+        <v>-0.08302071095901023</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>0.08216247475368543</v>
+        <v>0.08216247475368557</v>
       </c>
       <c r="M15" t="inlineStr">
         <is>
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>-0.08389513865189659</v>
+        <v>-0.08389513865189549</v>
       </c>
       <c r="O15" t="inlineStr">
         <is>
@@ -1659,7 +1659,7 @@
         </is>
       </c>
       <c r="P15" t="n">
-        <v>0.09910467858627972</v>
+        <v>0.0991046785862803</v>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="R15" t="n">
-        <v>0.08619939066437056</v>
+        <v>0.08619939066437039</v>
       </c>
       <c r="S15" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
         </is>
       </c>
       <c r="T15" t="n">
-        <v>-0.09883501297721427</v>
+        <v>-0.09883501297721442</v>
       </c>
     </row>
     <row r="16">
@@ -1685,7 +1685,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>0.05319545564918726</v>
+        <v>0.05319545564918724</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1693,7 +1693,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.05790141379377656</v>
+        <v>0.05790141379377652</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -1701,7 +1701,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.06145097787219254</v>
+        <v>0.06145097787219239</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -1717,7 +1717,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>0.08208524844328795</v>
+        <v>0.08208524844328792</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1733,7 +1733,7 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>-0.08052852892396567</v>
+        <v>-0.08052852892396553</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
@@ -1741,7 +1741,7 @@
         </is>
       </c>
       <c r="P16" t="n">
-        <v>-0.09756795951870462</v>
+        <v>-0.09756795951870463</v>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
@@ -1749,7 +1749,7 @@
         </is>
       </c>
       <c r="R16" t="n">
-        <v>0.08507389289251595</v>
+        <v>0.08507389289251631</v>
       </c>
       <c r="S16" t="inlineStr">
         <is>
@@ -1757,7 +1757,7 @@
         </is>
       </c>
       <c r="T16" t="n">
-        <v>0.09758736872364442</v>
+        <v>0.09758736872364449</v>
       </c>
     </row>
     <row r="17">
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>0.05319470845188428</v>
+        <v>0.05319470845188429</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1775,7 +1775,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.05779788132029856</v>
+        <v>0.05779788132029846</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1783,7 +1783,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.06143587678167639</v>
+        <v>0.06143587678167629</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -1791,7 +1791,7 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>0.07045242265341869</v>
+        <v>0.07045242265341872</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>-0.08064948077151525</v>
+        <v>-0.08064948077151518</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1807,7 +1807,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>-0.08115329373106532</v>
+        <v>-0.0811532937310654</v>
       </c>
       <c r="M17" t="inlineStr">
         <is>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>0.07838988318418236</v>
+        <v>0.07838988318418202</v>
       </c>
       <c r="O17" t="inlineStr">
         <is>
@@ -1823,7 +1823,7 @@
         </is>
       </c>
       <c r="P17" t="n">
-        <v>-0.09430820129487491</v>
+        <v>-0.09430820129487548</v>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
@@ -1831,7 +1831,7 @@
         </is>
       </c>
       <c r="R17" t="n">
-        <v>-0.08493749120220222</v>
+        <v>-0.08493749120220248</v>
       </c>
       <c r="S17" t="inlineStr">
         <is>
@@ -1839,7 +1839,7 @@
         </is>
       </c>
       <c r="T17" t="n">
-        <v>0.09758640281115422</v>
+        <v>0.09758640281115404</v>
       </c>
     </row>
     <row r="18">
@@ -1849,7 +1849,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>0.05316091614912957</v>
+        <v>0.05316091614912953</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1857,7 +1857,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.05766833809802152</v>
+        <v>0.05766833809802143</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1865,7 +1865,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.06091026899112802</v>
+        <v>0.06091026899112791</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -1873,7 +1873,7 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>0.07043148827440883</v>
+        <v>0.07043148827440888</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>0.0803125893210552</v>
+        <v>0.08031258932105528</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1897,7 +1897,7 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>0.0775160669948621</v>
+        <v>0.07751606699486208</v>
       </c>
       <c r="O18" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="P18" t="n">
-        <v>-0.09429197758624501</v>
+        <v>-0.09429197758624508</v>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
@@ -1913,7 +1913,7 @@
         </is>
       </c>
       <c r="R18" t="n">
-        <v>-0.08473549701004859</v>
+        <v>-0.08473549701004843</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -1921,7 +1921,7 @@
         </is>
       </c>
       <c r="T18" t="n">
-        <v>0.09585745433818413</v>
+        <v>0.0958574543381838</v>
       </c>
     </row>
     <row r="19">
@@ -1931,7 +1931,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>0.05311592282279368</v>
+        <v>0.05311592282279366</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1939,7 +1939,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.05763468692970023</v>
+        <v>0.05763468692970016</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1947,7 +1947,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.06073370723676565</v>
+        <v>0.06073370723676554</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1955,7 +1955,7 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>0.07001146010084915</v>
+        <v>0.0700114601008491</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1963,7 +1963,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>0.07856576146106603</v>
+        <v>0.0785657614610661</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>-0.07883372782165911</v>
+        <v>-0.07883372782165912</v>
       </c>
       <c r="M19" t="inlineStr">
         <is>
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>0.07747584957878532</v>
+        <v>0.07747584957878501</v>
       </c>
       <c r="O19" t="inlineStr">
         <is>
@@ -1987,7 +1987,7 @@
         </is>
       </c>
       <c r="P19" t="n">
-        <v>-0.09332706628224716</v>
+        <v>-0.09332706628224732</v>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="R19" t="n">
-        <v>0.08442659166209704</v>
+        <v>0.08442659166209703</v>
       </c>
       <c r="S19" t="inlineStr">
         <is>
@@ -2003,7 +2003,7 @@
         </is>
       </c>
       <c r="T19" t="n">
-        <v>-0.09411370243043991</v>
+        <v>-0.09411370243043983</v>
       </c>
     </row>
     <row r="20">
@@ -2013,7 +2013,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>0.05306402173415983</v>
+        <v>0.05306402173415979</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2021,7 +2021,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.05752757817345197</v>
+        <v>0.05752757817345189</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.06067821132757273</v>
+        <v>0.06067821132757267</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>0.0695907085727135</v>
+        <v>0.06959070857271353</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>-0.07698124722749669</v>
+        <v>-0.07698124722749675</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -2053,7 +2053,7 @@
         </is>
       </c>
       <c r="L20" t="n">
-        <v>-0.07754326185887049</v>
+        <v>-0.07754326185887053</v>
       </c>
       <c r="M20" t="inlineStr">
         <is>
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>0.07704568096546446</v>
+        <v>0.0770456809654642</v>
       </c>
       <c r="O20" t="inlineStr">
         <is>
@@ -2069,7 +2069,7 @@
         </is>
       </c>
       <c r="P20" t="n">
-        <v>-0.0930554269514374</v>
+        <v>-0.09305542695143769</v>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
@@ -2077,7 +2077,7 @@
         </is>
       </c>
       <c r="R20" t="n">
-        <v>0.08316156084794891</v>
+        <v>0.08316156084794869</v>
       </c>
       <c r="S20" t="inlineStr">
         <is>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="T20" t="n">
-        <v>-0.09283096836579435</v>
+        <v>-0.09283096836579451</v>
       </c>
     </row>
     <row r="21">
@@ -2095,7 +2095,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>0.05302922557402437</v>
+        <v>0.05302922557402438</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2103,7 +2103,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.05751596064026176</v>
+        <v>0.05751596064026167</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2111,7 +2111,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.0606265650303966</v>
+        <v>0.06062656503039653</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -2119,7 +2119,7 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>-0.06957886060265489</v>
+        <v>-0.06957886060265478</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -2127,7 +2127,7 @@
         </is>
       </c>
       <c r="J21" t="n">
-        <v>-0.0765849710162344</v>
+        <v>-0.07658497101623442</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="L21" t="n">
-        <v>-0.07752631395412245</v>
+        <v>-0.07752631395412243</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -2143,7 +2143,7 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>0.076623551716317</v>
+        <v>0.07662355171631711</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
@@ -2151,7 +2151,7 @@
         </is>
       </c>
       <c r="P21" t="n">
-        <v>-0.09298266753015501</v>
+        <v>-0.09298266753015515</v>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
@@ -2159,7 +2159,7 @@
         </is>
       </c>
       <c r="R21" t="n">
-        <v>0.08153118793945723</v>
+        <v>0.08153118793945692</v>
       </c>
       <c r="S21" t="inlineStr">
         <is>
@@ -2167,7 +2167,7 @@
         </is>
       </c>
       <c r="T21" t="n">
-        <v>-0.08951529269046801</v>
+        <v>-0.08951529269046825</v>
       </c>
     </row>
   </sheetData>

</xml_diff>